<commit_message>
Wifi RGB LCD Board BOM updated.
</commit_message>
<xml_diff>
--- a/Design-Files/WIFI_Board_RGB-LCDV4.0/BOM/Client-BOM-WIFI_BoardV4.10.xlsx
+++ b/Design-Files/WIFI_Board_RGB-LCDV4.0/BOM/Client-BOM-WIFI_BoardV4.10.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="305">
   <si>
     <t>#</t>
   </si>
@@ -919,6 +919,21 @@
   </si>
   <si>
     <t>Order LCD Without touch panel</t>
+  </si>
+  <si>
+    <t>Q6</t>
+  </si>
+  <si>
+    <t>30V 5.8A 32mΩ@10V,5.8A 1.4W 1.4V@250uA 1 N-Channel SOT-23 MOSFETs ROHS</t>
+  </si>
+  <si>
+    <t>SOT-24</t>
+  </si>
+  <si>
+    <t>AO3400A</t>
+  </si>
+  <si>
+    <t>BORN</t>
   </si>
 </sst>
 </file>
@@ -1147,9 +1162,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1161,6 +1173,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1450,7 +1465,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1474,9 +1489,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1546,7 +1561,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B62" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B63" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -2416,28 +2431,28 @@
       <c r="C31" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="F31" s="15" t="s">
+      <c r="F31" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="G31" s="15" t="s">
+      <c r="G31" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="H31" s="15" t="s">
+      <c r="H31" s="14" t="s">
         <v>293</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="14">
         <v>5</v>
       </c>
-      <c r="K31" s="17" t="s">
+      <c r="K31" s="16" t="s">
         <v>294</v>
       </c>
     </row>
@@ -2505,992 +2520,1023 @@
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
-        <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="I34" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="J34" s="9">
-        <v>4</v>
-      </c>
-      <c r="K34" s="9"/>
+      <c r="C34" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="J34" s="7">
+        <v>1</v>
+      </c>
+      <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
-        <f>ROW(B35) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="I35" s="8" t="s">
+      <c r="D35" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="I35" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="J35" s="7">
-        <v>2</v>
-      </c>
-      <c r="K35" s="7"/>
+      <c r="J35" s="9">
+        <v>4</v>
+      </c>
+      <c r="K35" s="9"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="F36" s="9" t="s">
+      <c r="D36" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G36" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="J36" s="9">
-        <v>10</v>
-      </c>
-      <c r="K36" s="9"/>
+      <c r="G36" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="J36" s="7">
+        <v>2</v>
+      </c>
+      <c r="K36" s="7"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
-        <f>ROW(B37) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="F37" s="7" t="s">
+      <c r="D37" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="F37" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G37" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="H37" s="7" t="s">
+      <c r="G37" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I37" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="J37" s="7">
-        <v>3</v>
-      </c>
-      <c r="K37" s="7"/>
+      <c r="I37" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="J37" s="9">
+        <v>10</v>
+      </c>
+      <c r="K37" s="9"/>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B38) - ROW($B$2)</f>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D38" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="F38" s="9" t="s">
+      <c r="D38" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="F38" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G38" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H38" s="9" t="s">
+      <c r="G38" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="H38" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I38" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="J38" s="9">
-        <v>6</v>
-      </c>
-      <c r="K38" s="9"/>
-    </row>
-    <row r="39" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I38" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="J38" s="7">
+        <v>3</v>
+      </c>
+      <c r="K38" s="7"/>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
-        <f>ROW(B39) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C39" s="12" t="s">
+      <c r="C39" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="J39" s="7">
-        <v>1</v>
-      </c>
-      <c r="K39" s="7"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D39" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="J39" s="9">
+        <v>6</v>
+      </c>
+      <c r="K39" s="9"/>
+    </row>
+    <row r="40" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$2)</f>
         <v>38</v>
       </c>
-      <c r="C40" s="13" t="s">
+      <c r="C40" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="I40" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="J40" s="9">
-        <v>2</v>
-      </c>
-      <c r="K40" s="9"/>
+      <c r="D40" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="J40" s="7">
+        <v>1</v>
+      </c>
+      <c r="K40" s="7"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
-        <f>ROW(B41) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="H41" s="7" t="s">
+      <c r="D41" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I41" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="J41" s="7">
-        <v>1</v>
-      </c>
-      <c r="K41" s="7"/>
+      <c r="I41" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="J41" s="9">
+        <v>2</v>
+      </c>
+      <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B42) - ROW($B$2)</f>
         <v>40</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F42" s="9" t="s">
+      <c r="D42" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F42" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="G42" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H42" s="9" t="s">
+      <c r="G42" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="H42" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I42" s="10" t="s">
-        <v>280</v>
-      </c>
-      <c r="J42" s="9">
-        <v>1</v>
-      </c>
-      <c r="K42" s="9"/>
+      <c r="I42" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="J42" s="7">
+        <v>1</v>
+      </c>
+      <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
-        <f>ROW(B43) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C43" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F43" s="7" t="s">
+      <c r="C43" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F43" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="G43" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="H43" s="7" t="s">
+      <c r="G43" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I43" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="J43" s="7">
-        <v>1</v>
-      </c>
-      <c r="K43" s="7"/>
+      <c r="I43" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="J43" s="9">
+        <v>1</v>
+      </c>
+      <c r="K43" s="9"/>
     </row>
     <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B44) - ROW($B$2)</f>
         <v>42</v>
       </c>
-      <c r="C44" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F44" s="9" t="s">
+      <c r="C44" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F44" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="G44" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="H44" s="9" t="s">
+      <c r="G44" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="H44" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I44" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="J44" s="9">
-        <v>2</v>
-      </c>
-      <c r="K44" s="9"/>
+      <c r="I44" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="J44" s="7">
+        <v>1</v>
+      </c>
+      <c r="K44" s="7"/>
     </row>
     <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
-        <f>ROW(B45) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="F45" s="7" t="s">
+      <c r="D45" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F45" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="G45" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="H45" s="7" t="s">
+      <c r="G45" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I45" s="8" t="s">
-        <v>282</v>
-      </c>
-      <c r="J45" s="7">
+      <c r="I45" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="J45" s="9">
         <v>2</v>
       </c>
-      <c r="K45" s="7"/>
+      <c r="K45" s="9"/>
     </row>
     <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B46) - ROW($B$2)</f>
         <v>44</v>
       </c>
-      <c r="C46" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="G46" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="H46" s="9" t="s">
+      <c r="C46" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="H46" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I46" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="J46" s="9">
+      <c r="I46" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="J46" s="7">
         <v>2</v>
       </c>
-      <c r="K46" s="9"/>
+      <c r="K46" s="7"/>
     </row>
     <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
-        <f>ROW(B47) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="C47" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="F47" s="7" t="s">
+      <c r="C47" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="F47" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G47" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="H47" s="7" t="s">
+      <c r="G47" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="H47" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I47" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="J47" s="7">
-        <v>1</v>
-      </c>
-      <c r="K47" s="7"/>
+      <c r="I47" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="J47" s="9">
+        <v>2</v>
+      </c>
+      <c r="K47" s="9"/>
     </row>
     <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B48) - ROW($B$2)</f>
         <v>46</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="F48" s="9" t="s">
+      <c r="D48" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="F48" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G48" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="H48" s="9" t="s">
+      <c r="G48" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="H48" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I48" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="J48" s="9">
-        <v>1</v>
-      </c>
-      <c r="K48" s="9"/>
+      <c r="I48" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="J48" s="7">
+        <v>1</v>
+      </c>
+      <c r="K48" s="7"/>
     </row>
     <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
-        <f>ROW(B49) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="C49" s="12" t="s">
+      <c r="C49" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D49" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="F49" s="7" t="s">
+      <c r="D49" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F49" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G49" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="I49" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="J49" s="7">
-        <v>4</v>
-      </c>
-      <c r="K49" s="7"/>
+      <c r="G49" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="J49" s="9">
+        <v>1</v>
+      </c>
+      <c r="K49" s="9"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B50) - ROW($B$2)</f>
         <v>48</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="C50" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="F50" s="9" t="s">
+      <c r="D50" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F50" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G50" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="H50" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>286</v>
-      </c>
-      <c r="J50" s="9">
-        <v>2</v>
-      </c>
-      <c r="K50" s="9"/>
+      <c r="G50" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="J50" s="7">
+        <v>4</v>
+      </c>
+      <c r="K50" s="7"/>
     </row>
     <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
-        <f>ROW(B51) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="C51" s="12" t="s">
+      <c r="C51" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D51" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F51" s="7" t="s">
+      <c r="D51" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G51" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="H51" s="7" t="s">
+      <c r="G51" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="H51" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I51" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="J51" s="7">
-        <v>1</v>
-      </c>
-      <c r="K51" s="7"/>
+      <c r="I51" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J51" s="9">
+        <v>2</v>
+      </c>
+      <c r="K51" s="9"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B52) - ROW($B$2)</f>
         <v>50</v>
       </c>
-      <c r="C52" s="13" t="s">
+      <c r="C52" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="H52" s="9" t="s">
+      <c r="D52" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="H52" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="I52" s="10" t="s">
-        <v>286</v>
-      </c>
-      <c r="J52" s="9">
-        <v>2</v>
-      </c>
-      <c r="K52" s="9"/>
+      <c r="I52" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="J52" s="7">
+        <v>1</v>
+      </c>
+      <c r="K52" s="7"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
-        <f>ROW(B53) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>137</v>
+      <c r="C53" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="H53" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="I53" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="J53" s="7">
+        <v>164</v>
+      </c>
+      <c r="G53" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J53" s="9">
         <v>2</v>
       </c>
-      <c r="K53" s="7"/>
+      <c r="K53" s="9"/>
     </row>
     <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B54) - ROW($B$2)</f>
         <v>52</v>
       </c>
-      <c r="C54" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D54" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>138</v>
+      <c r="C54" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="G54" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>254</v>
+      <c r="G54" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="H54" s="7" t="s">
+        <v>253</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J54" s="9">
-        <v>1</v>
-      </c>
-      <c r="K54" s="9"/>
+      <c r="J54" s="7">
+        <v>2</v>
+      </c>
+      <c r="K54" s="7"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f>ROW(B55) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="C55" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>137</v>
+      <c r="C55" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>138</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="G55" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="H55" s="7" t="s">
-        <v>255</v>
+      <c r="G55" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>254</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J55" s="7">
-        <v>3</v>
-      </c>
-      <c r="K55" s="7"/>
+      <c r="J55" s="9">
+        <v>1</v>
+      </c>
+      <c r="K55" s="9"/>
     </row>
     <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B56) - ROW($B$2)</f>
         <v>54</v>
       </c>
-      <c r="C56" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>139</v>
+      <c r="C56" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="G56" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="H56" s="9" t="s">
-        <v>256</v>
+        <v>295</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>255</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J56" s="9">
-        <v>1</v>
-      </c>
-      <c r="K56" s="9"/>
-    </row>
-    <row r="57" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J56" s="7">
+        <v>3</v>
+      </c>
+      <c r="K56" s="7"/>
+    </row>
+    <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
-        <f>ROW(B57) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="C57" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>140</v>
+      <c r="C57" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="G57" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>257</v>
+        <v>169</v>
+      </c>
+      <c r="G57" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>256</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J57" s="7">
-        <v>1</v>
-      </c>
-      <c r="K57" s="7"/>
-    </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J57" s="9">
+        <v>1</v>
+      </c>
+      <c r="K57" s="9"/>
+    </row>
+    <row r="58" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B58) - ROW($B$2)</f>
         <v>56</v>
       </c>
-      <c r="C58" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>141</v>
+      <c r="C58" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>140</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>258</v>
+        <v>295</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>257</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J58" s="9">
-        <v>1</v>
-      </c>
-      <c r="K58" s="9"/>
-    </row>
-    <row r="59" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J58" s="7">
+        <v>1</v>
+      </c>
+      <c r="K58" s="7"/>
+    </row>
+    <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
-        <f>ROW(B59) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="G59" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>259</v>
+      <c r="C59" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="G59" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>258</v>
       </c>
       <c r="I59" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J59" s="7">
-        <v>1</v>
-      </c>
-      <c r="K59" s="7"/>
-    </row>
-    <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J59" s="9">
+        <v>1</v>
+      </c>
+      <c r="K59" s="9"/>
+    </row>
+    <row r="60" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B60) - ROW($B$2)</f>
         <v>58</v>
       </c>
-      <c r="C60" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D60" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="G60" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="H60" s="9" t="s">
-        <v>260</v>
+      <c r="C60" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>259</v>
       </c>
       <c r="I60" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J60" s="9">
-        <v>1</v>
-      </c>
-      <c r="K60" s="9"/>
-    </row>
-    <row r="61" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J60" s="7">
+        <v>1</v>
+      </c>
+      <c r="K60" s="7"/>
+    </row>
+    <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
-        <f>ROW(B61) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="C61" s="12" t="s">
+      <c r="C61" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D61" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="H61" s="7" t="s">
-        <v>261</v>
+      <c r="D61" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="G61" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>260</v>
       </c>
       <c r="I61" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J61" s="7">
-        <v>1</v>
-      </c>
-      <c r="K61" s="7"/>
-    </row>
-    <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J61" s="9">
+        <v>1</v>
+      </c>
+      <c r="K61" s="9"/>
+    </row>
+    <row r="62" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B62) - ROW($B$2)</f>
         <v>60</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D62" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="F62" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="G62" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="H62" s="9" t="s">
-        <v>262</v>
+      <c r="D62" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>261</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="J62" s="9">
-        <v>1</v>
-      </c>
-      <c r="K62" s="9"/>
-    </row>
-    <row r="63" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J62" s="7">
+        <v>1</v>
+      </c>
+      <c r="K62" s="7"/>
+    </row>
+    <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
-        <f>ROW(B63) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C63" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D63" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="F63" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>263</v>
+      <c r="C63" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G63" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>262</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="J63" s="7">
-        <v>1</v>
-      </c>
-      <c r="K63" s="7"/>
-    </row>
-    <row r="64" spans="1:11" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+      <c r="J63" s="9">
+        <v>1</v>
+      </c>
+      <c r="K63" s="9"/>
+    </row>
+    <row r="64" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="1"/>
       <c r="B64" s="11">
         <f>ROW(B64) - ROW($B$2)</f>
         <v>62</v>
       </c>
       <c r="C64" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F64" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="H64" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I64" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="J64" s="7">
+        <v>1</v>
+      </c>
+      <c r="K64" s="7"/>
+    </row>
+    <row r="65" spans="2:11" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="11">
+        <f>ROW(B65) - ROW($B$2)</f>
+        <v>63</v>
+      </c>
+      <c r="C65" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="D64" s="7" t="s">
+      <c r="D65" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="E64" s="8" t="s">
+      <c r="E65" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="F64" s="7" t="s">
+      <c r="F65" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="G64" s="7" t="s">
+      <c r="G65" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="H64" s="7"/>
-      <c r="I64" s="8"/>
-      <c r="J64" s="7">
-        <v>1</v>
-      </c>
-      <c r="K64" s="18" t="s">
+      <c r="H65" s="7"/>
+      <c r="I65" s="8"/>
+      <c r="J65" s="7">
+        <v>1</v>
+      </c>
+      <c r="K65" s="17" t="s">
         <v>299</v>
       </c>
     </row>
@@ -3499,7 +3545,7 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K64" r:id="rId1"/>
+    <hyperlink ref="K65" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>